<commit_message>
Add editor/pyright venv config and update data template
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/SusTool_data_template.xlsx
+++ b/data/SusTool_data_template.xlsx
@@ -2327,16 +2327,16 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <u/>
       <sz val="11"/>
-      <color rgb="FF006100"/>
+      <color rgb="FF800080"/>
       <name val="等线"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
       <sz val="11"/>
-      <color rgb="FF800080"/>
+      <color rgb="FF006100"/>
       <name val="等线"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -2941,7 +2941,7 @@
     <xf numFmtId="0" fontId="21" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
@@ -3021,7 +3021,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="6"/>
@@ -3029,12 +3029,13 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="6" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="6" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="6" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="6" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="6" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -3070,21 +3071,21 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="22"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="22"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="22" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="22" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="6" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="22" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="22" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -3098,7 +3099,7 @@
     <xf numFmtId="0" fontId="7" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="22" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="22" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -3122,7 +3123,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="22" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" xfId="22" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -3490,62 +3491,62 @@
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelRow="1" outlineLevelCol="7"/>
   <cols>
-    <col min="1" max="1" width="12.0892857142857" style="25" customWidth="1"/>
-    <col min="2" max="2" width="10.4553571428571" style="25" customWidth="1"/>
-    <col min="3" max="5" width="8.72321428571429" style="41"/>
-    <col min="6" max="7" width="8.72321428571429" style="25"/>
+    <col min="1" max="1" width="12.0892857142857" style="26" customWidth="1"/>
+    <col min="2" max="2" width="10.4553571428571" style="26" customWidth="1"/>
+    <col min="3" max="5" width="8.72321428571429" style="42"/>
+    <col min="6" max="7" width="8.72321428571429" style="26"/>
     <col min="8" max="8" width="96.3660714285714" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="31" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="30" t="s">
+      <c r="B1" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="40" t="s">
+      <c r="C1" s="41" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="40" t="s">
+      <c r="D1" s="41" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="40" t="s">
+      <c r="E1" s="41" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="48" t="s">
+      <c r="F1" s="49" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="30" t="s">
+      <c r="G1" s="31" t="s">
         <v>6</v>
       </c>
       <c r="H1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" s="46" customFormat="1" ht="77" customHeight="1" spans="1:8">
-      <c r="A2" s="25" t="s">
+    <row r="2" s="47" customFormat="1" ht="77" customHeight="1" spans="1:8">
+      <c r="A2" s="26" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="25" t="s">
+      <c r="B2" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="41">
+      <c r="C2" s="42">
         <v>3</v>
       </c>
-      <c r="D2" s="41">
+      <c r="D2" s="42">
         <v>1</v>
       </c>
-      <c r="E2" s="41">
+      <c r="E2" s="42">
         <v>5</v>
       </c>
-      <c r="F2" s="25">
+      <c r="F2" s="26">
         <v>7000</v>
       </c>
-      <c r="G2" s="25" t="s">
+      <c r="G2" s="26" t="s">
         <v>10</v>
       </c>
-      <c r="H2" s="47" t="s">
+      <c r="H2" s="48" t="s">
         <v>11</v>
       </c>
     </row>
@@ -3571,48 +3572,48 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="24" t="s">
+      <c r="B1" s="25" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="24" t="s">
+      <c r="C1" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="D1" s="24" t="s">
+      <c r="D1" s="25" t="s">
         <v>13</v>
       </c>
-      <c r="E1" s="24" t="s">
+      <c r="E1" s="25" t="s">
         <v>14</v>
       </c>
-      <c r="F1" s="24" t="s">
+      <c r="F1" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="G1" s="24" t="s">
+      <c r="G1" s="25" t="s">
         <v>6</v>
       </c>
       <c r="H1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="2" s="46" customFormat="1" ht="135" spans="1:8">
-      <c r="A2" s="46" t="s">
+    <row r="2" s="47" customFormat="1" ht="135" spans="1:8">
+      <c r="A2" s="47" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="46" t="s">
+      <c r="B2" s="47" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="46" t="s">
+      <c r="C2" s="47" t="s">
         <v>17</v>
       </c>
-      <c r="D2" s="46" t="s">
+      <c r="D2" s="47" t="s">
         <v>18</v>
       </c>
-      <c r="G2" s="46" t="s">
+      <c r="G2" s="47" t="s">
         <v>10</v>
       </c>
-      <c r="H2" s="47" t="s">
+      <c r="H2" s="48" t="s">
         <v>19</v>
       </c>
     </row>
@@ -3645,137 +3646,137 @@
   <dimension ref="A1:G8"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelRow="7" outlineLevelCol="6"/>
   <cols>
-    <col min="1" max="1" width="12.0892857142857" style="12" customWidth="1"/>
-    <col min="2" max="2" width="22.3660714285714" style="12" customWidth="1"/>
-    <col min="3" max="3" width="15.9107142857143" style="12" customWidth="1"/>
-    <col min="4" max="4" width="16.6339285714286" style="12" customWidth="1"/>
-    <col min="5" max="5" width="13.8125" style="12" customWidth="1"/>
-    <col min="6" max="6" width="7.63392857142857" style="12" customWidth="1"/>
+    <col min="1" max="1" width="12.0892857142857" style="13" customWidth="1"/>
+    <col min="2" max="2" width="22.3660714285714" style="13" customWidth="1"/>
+    <col min="3" max="3" width="15.9107142857143" style="13" customWidth="1"/>
+    <col min="4" max="4" width="16.6339285714286" style="13" customWidth="1"/>
+    <col min="5" max="5" width="13.8125" style="13" customWidth="1"/>
+    <col min="6" max="6" width="7.63392857142857" style="13" customWidth="1"/>
     <col min="7" max="7" width="79.3660714285714" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="40" t="s">
+      <c r="A1" s="41" t="s">
         <v>22</v>
       </c>
-      <c r="B1" s="40" t="s">
+      <c r="B1" s="41" t="s">
         <v>23</v>
       </c>
-      <c r="C1" s="40" t="s">
+      <c r="C1" s="41" t="s">
         <v>24</v>
       </c>
-      <c r="D1" s="40" t="s">
+      <c r="D1" s="41" t="s">
         <v>25</v>
       </c>
-      <c r="E1" s="40" t="s">
+      <c r="E1" s="41" t="s">
         <v>26</v>
       </c>
-      <c r="F1" s="40" t="s">
+      <c r="F1" s="41" t="s">
         <v>6</v>
       </c>
-      <c r="G1" s="42" t="s">
+      <c r="G1" s="43" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1" spans="1:7">
-      <c r="A2" s="41" t="s">
+      <c r="A2" s="42" t="s">
         <v>28</v>
       </c>
-      <c r="B2" s="41">
+      <c r="B2" s="42">
         <v>100</v>
       </c>
-      <c r="C2" s="41"/>
-      <c r="D2" s="41"/>
-      <c r="E2" s="41" t="s">
+      <c r="C2" s="42"/>
+      <c r="D2" s="42"/>
+      <c r="E2" s="42" t="s">
         <v>29</v>
       </c>
-      <c r="F2" s="41" t="s">
+      <c r="F2" s="42" t="s">
         <v>10</v>
       </c>
-      <c r="G2" s="43" t="s">
+      <c r="G2" s="44" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="3" ht="17" spans="1:7">
-      <c r="A3" s="41" t="s">
+      <c r="A3" s="42" t="s">
         <v>31</v>
       </c>
-      <c r="B3" s="41">
+      <c r="B3" s="42">
         <v>1000</v>
       </c>
-      <c r="C3" s="41"/>
-      <c r="D3" s="41"/>
-      <c r="E3" s="41" t="s">
+      <c r="C3" s="42"/>
+      <c r="D3" s="42"/>
+      <c r="E3" s="42" t="s">
         <v>32</v>
       </c>
-      <c r="F3" s="41" t="s">
+      <c r="F3" s="42" t="s">
         <v>10</v>
       </c>
-      <c r="G3" s="43" t="s">
+      <c r="G3" s="44" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="4" spans="1:7">
-      <c r="A4" s="41" t="s">
+      <c r="A4" s="42" t="s">
         <v>34</v>
       </c>
-      <c r="B4" s="41" t="s">
+      <c r="B4" s="42" t="s">
         <v>35</v>
       </c>
-      <c r="C4" s="41"/>
-      <c r="D4" s="41"/>
-      <c r="E4" s="41" t="s">
+      <c r="C4" s="42"/>
+      <c r="D4" s="42"/>
+      <c r="E4" s="42" t="s">
         <v>29</v>
       </c>
-      <c r="F4" s="41" t="s">
+      <c r="F4" s="42" t="s">
         <v>10</v>
       </c>
-      <c r="G4" s="44" t="s">
+      <c r="G4" s="45" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="5" ht="118" spans="1:7">
-      <c r="A5" s="41" t="s">
+      <c r="A5" s="42" t="s">
         <v>37</v>
       </c>
-      <c r="B5" s="41">
+      <c r="B5" s="42">
         <v>1</v>
       </c>
-      <c r="C5" s="41"/>
-      <c r="D5" s="41"/>
-      <c r="E5" s="41" t="s">
+      <c r="C5" s="42"/>
+      <c r="D5" s="42"/>
+      <c r="E5" s="42" t="s">
         <v>32</v>
       </c>
-      <c r="F5" s="41" t="s">
+      <c r="F5" s="42" t="s">
         <v>10</v>
       </c>
-      <c r="G5" s="45" t="s">
+      <c r="G5" s="46" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="6" spans="1:6">
-      <c r="A6" s="41" t="s">
+      <c r="A6" s="42" t="s">
         <v>31</v>
       </c>
-      <c r="B6" s="41">
+      <c r="B6" s="42">
         <v>500</v>
       </c>
-      <c r="C6" s="41"/>
-      <c r="D6" s="41"/>
-      <c r="E6" s="41" t="s">
+      <c r="C6" s="42"/>
+      <c r="D6" s="42"/>
+      <c r="E6" s="42" t="s">
         <v>39</v>
       </c>
-      <c r="F6" s="41" t="s">
+      <c r="F6" s="42" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="7" spans="5:5">
-      <c r="E7" s="12" t="s">
+      <c r="E7" s="13" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="8" spans="5:5">
-      <c r="E8" s="12" t="s">
+      <c r="E8" s="13" t="s">
         <v>42</v>
       </c>
     </row>
@@ -3859,8 +3860,8 @@
       <c r="H1" t="s">
         <v>52</v>
       </c>
-      <c r="K1" s="33"/>
-      <c r="L1" s="34" t="s">
+      <c r="K1" s="34"/>
+      <c r="L1" s="35" t="s">
         <v>53</v>
       </c>
       <c r="N1" s="1" t="s">
@@ -3890,10 +3891,10 @@
         <v>59</v>
       </c>
       <c r="J2" s="2"/>
-      <c r="K2" s="33">
+      <c r="K2" s="34">
         <v>1</v>
       </c>
-      <c r="L2" s="33" t="s">
+      <c r="L2" s="34" t="s">
         <v>60</v>
       </c>
     </row>
@@ -3919,10 +3920,10 @@
       <c r="H3" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="K3" s="33">
+      <c r="K3" s="34">
         <v>2</v>
       </c>
-      <c r="L3" s="33" t="s">
+      <c r="L3" s="34" t="s">
         <v>67</v>
       </c>
     </row>
@@ -3945,13 +3946,13 @@
       <c r="G4" t="s">
         <v>72</v>
       </c>
-      <c r="H4" s="38" t="s">
+      <c r="H4" s="39" t="s">
         <v>73</v>
       </c>
-      <c r="K4" s="33">
+      <c r="K4" s="34">
         <v>3</v>
       </c>
-      <c r="L4" s="33" t="s">
+      <c r="L4" s="34" t="s">
         <v>74</v>
       </c>
     </row>
@@ -3974,13 +3975,13 @@
       <c r="G5" t="s">
         <v>79</v>
       </c>
-      <c r="K5" s="33">
+      <c r="K5" s="34">
         <v>4</v>
       </c>
-      <c r="L5" s="33" t="s">
+      <c r="L5" s="34" t="s">
         <v>80</v>
       </c>
-      <c r="P5" s="39"/>
+      <c r="P5" s="40"/>
     </row>
     <row r="6" spans="1:8">
       <c r="A6">
@@ -4302,7 +4303,7 @@
       <c r="A20">
         <v>16</v>
       </c>
-      <c r="B20" s="37" t="s">
+      <c r="B20" s="38" t="s">
         <v>132</v>
       </c>
       <c r="C20" t="s">
@@ -5440,11 +5441,11 @@
   <cols>
     <col min="1" max="1" width="3.17857142857143" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="3" max="3" width="24.1785714285714" style="12" customWidth="1"/>
+    <col min="3" max="3" width="24.1785714285714" style="13" customWidth="1"/>
     <col min="4" max="5" width="39.6339285714286" customWidth="1"/>
     <col min="6" max="6" width="15.3660714285714" customWidth="1"/>
-    <col min="7" max="8" width="15.2678571428571" style="25" customWidth="1"/>
-    <col min="9" max="9" width="19.9107142857143" style="12" customWidth="1"/>
+    <col min="7" max="8" width="15.2678571428571" style="26" customWidth="1"/>
+    <col min="9" max="9" width="19.9107142857143" style="13" customWidth="1"/>
     <col min="10" max="10" width="5.54464285714286" customWidth="1"/>
     <col min="12" max="12" width="3.17857142857143" customWidth="1"/>
     <col min="13" max="13" width="3.26785714285714" customWidth="1"/>
@@ -5453,35 +5454,35 @@
     <col min="17" max="17" width="13.2678571428571" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="24" customFormat="1" spans="2:11">
-      <c r="B1" s="24" t="s">
+    <row r="1" s="25" customFormat="1" spans="2:11">
+      <c r="B1" s="25" t="s">
         <v>43</v>
       </c>
-      <c r="C1" s="26" t="s">
+      <c r="C1" s="27" t="s">
         <v>264</v>
       </c>
-      <c r="D1" s="24" t="s">
+      <c r="D1" s="25" t="s">
         <v>265</v>
       </c>
-      <c r="E1" s="24" t="s">
+      <c r="E1" s="25" t="s">
         <v>266</v>
       </c>
-      <c r="F1" s="24" t="s">
+      <c r="F1" s="25" t="s">
         <v>267</v>
       </c>
-      <c r="G1" s="30" t="s">
+      <c r="G1" s="31" t="s">
         <v>268</v>
       </c>
-      <c r="H1" s="30" t="s">
+      <c r="H1" s="31" t="s">
         <v>269</v>
       </c>
-      <c r="I1" s="26" t="s">
+      <c r="I1" s="27" t="s">
         <v>270</v>
       </c>
-      <c r="J1" s="24" t="s">
+      <c r="J1" s="25" t="s">
         <v>271</v>
       </c>
-      <c r="K1" s="24" t="s">
+      <c r="K1" s="25" t="s">
         <v>272</v>
       </c>
     </row>
@@ -5492,20 +5493,20 @@
       <c r="B2" t="s">
         <v>273</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="C2" s="13" t="s">
         <v>274</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>275</v>
       </c>
       <c r="E2" s="2"/>
-      <c r="G2" s="25">
+      <c r="G2" s="26">
         <v>450</v>
       </c>
-      <c r="H2" s="25">
+      <c r="H2" s="26">
         <v>38</v>
       </c>
-      <c r="I2" s="12" t="s">
+      <c r="I2" s="13" t="s">
         <v>276</v>
       </c>
     </row>
@@ -5516,17 +5517,17 @@
       <c r="B3" t="s">
         <v>277</v>
       </c>
-      <c r="C3" s="12" t="s">
+      <c r="C3" s="13" t="s">
         <v>278</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>279</v>
       </c>
       <c r="E3" s="2"/>
-      <c r="H3" s="25">
+      <c r="H3" s="26">
         <v>39</v>
       </c>
-      <c r="I3" s="12" t="s">
+      <c r="I3" s="13" t="s">
         <v>280</v>
       </c>
     </row>
@@ -5537,7 +5538,7 @@
       <c r="B4" t="s">
         <v>281</v>
       </c>
-      <c r="C4" s="27">
+      <c r="C4" s="28">
         <v>0.32</v>
       </c>
       <c r="D4" s="2" t="s">
@@ -5547,13 +5548,13 @@
       <c r="F4" t="s">
         <v>283</v>
       </c>
-      <c r="G4" s="25">
+      <c r="G4" s="26">
         <v>400</v>
       </c>
-      <c r="H4" s="25">
+      <c r="H4" s="26">
         <v>32</v>
       </c>
-      <c r="I4" s="12" t="s">
+      <c r="I4" s="13" t="s">
         <v>284</v>
       </c>
       <c r="J4" t="s">
@@ -5567,20 +5568,20 @@
       <c r="B5" t="s">
         <v>286</v>
       </c>
-      <c r="C5" s="27" t="s">
+      <c r="C5" s="28" t="s">
         <v>287</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>282</v>
       </c>
       <c r="E5" s="2"/>
-      <c r="G5" s="25" t="s">
+      <c r="G5" s="26" t="s">
         <v>288</v>
       </c>
-      <c r="H5" s="25" t="s">
+      <c r="H5" s="26" t="s">
         <v>289</v>
       </c>
-      <c r="I5" s="12" t="s">
+      <c r="I5" s="13" t="s">
         <v>284</v>
       </c>
       <c r="J5" t="s">
@@ -5597,10 +5598,10 @@
       <c r="B6" t="s">
         <v>291</v>
       </c>
-      <c r="C6" s="12" t="s">
+      <c r="C6" s="13" t="s">
         <v>292</v>
       </c>
-      <c r="D6" s="28" t="s">
+      <c r="D6" s="29" t="s">
         <v>293</v>
       </c>
       <c r="E6" s="2" t="s">
@@ -5609,24 +5610,24 @@
       <c r="F6" t="s">
         <v>295</v>
       </c>
-      <c r="G6" s="25">
+      <c r="G6" s="26">
         <v>500</v>
       </c>
-      <c r="H6" s="11" t="s">
+      <c r="H6" s="12" t="s">
         <v>296</v>
       </c>
-      <c r="I6" s="12" t="s">
+      <c r="I6" s="13" t="s">
         <v>280</v>
       </c>
       <c r="M6" s="4"/>
       <c r="N6" s="4" t="s">
         <v>297</v>
       </c>
-      <c r="O6" s="33"/>
-      <c r="P6" s="34" t="s">
+      <c r="O6" s="34"/>
+      <c r="P6" s="35" t="s">
         <v>298</v>
       </c>
-      <c r="Q6" s="32" t="s">
+      <c r="Q6" s="33" t="s">
         <v>299</v>
       </c>
     </row>
@@ -5637,20 +5638,20 @@
       <c r="B7" t="s">
         <v>300</v>
       </c>
-      <c r="C7" s="27">
+      <c r="C7" s="28">
         <v>0.3</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>293</v>
       </c>
       <c r="E7" s="2"/>
-      <c r="G7" s="25">
+      <c r="G7" s="26">
         <v>500</v>
       </c>
-      <c r="H7" s="11">
+      <c r="H7" s="12">
         <v>30</v>
       </c>
-      <c r="I7" s="12" t="s">
+      <c r="I7" s="13" t="s">
         <v>280</v>
       </c>
       <c r="M7" s="4">
@@ -5659,13 +5660,13 @@
       <c r="N7" s="4" t="s">
         <v>301</v>
       </c>
-      <c r="O7" s="33">
+      <c r="O7" s="34">
         <v>1</v>
       </c>
-      <c r="P7" s="33" t="s">
+      <c r="P7" s="34" t="s">
         <v>302</v>
       </c>
-      <c r="Q7" s="32" t="s">
+      <c r="Q7" s="33" t="s">
         <v>217</v>
       </c>
     </row>
@@ -5676,20 +5677,20 @@
       <c r="B8" t="s">
         <v>303</v>
       </c>
-      <c r="C8" s="27">
+      <c r="C8" s="28">
         <v>0.32</v>
       </c>
-      <c r="D8" s="28" t="s">
+      <c r="D8" s="29" t="s">
         <v>293</v>
       </c>
       <c r="E8" s="2"/>
-      <c r="G8" s="25">
+      <c r="G8" s="26">
         <v>500</v>
       </c>
-      <c r="H8" s="11">
+      <c r="H8" s="12">
         <v>32</v>
       </c>
-      <c r="I8" s="12" t="s">
+      <c r="I8" s="13" t="s">
         <v>280</v>
       </c>
       <c r="M8" s="4">
@@ -5698,18 +5699,18 @@
       <c r="N8" s="4" t="s">
         <v>304</v>
       </c>
-      <c r="O8" s="33">
+      <c r="O8" s="34">
         <v>2</v>
       </c>
-      <c r="P8" s="33" t="s">
+      <c r="P8" s="34" t="s">
         <v>305</v>
       </c>
-      <c r="Q8" s="32" t="s">
+      <c r="Q8" s="33" t="s">
         <v>217</v>
       </c>
     </row>
     <row r="9" spans="3:17">
-      <c r="C9" s="12" t="s">
+      <c r="C9" s="13" t="s">
         <v>306</v>
       </c>
       <c r="D9" s="2" t="s">
@@ -5722,13 +5723,13 @@
       <c r="N9" s="4" t="s">
         <v>308</v>
       </c>
-      <c r="O9" s="33">
+      <c r="O9" s="34">
         <v>3</v>
       </c>
-      <c r="P9" s="33" t="s">
+      <c r="P9" s="34" t="s">
         <v>309</v>
       </c>
-      <c r="Q9" s="32" t="s">
+      <c r="Q9" s="33" t="s">
         <v>310</v>
       </c>
     </row>
@@ -5739,7 +5740,7 @@
       <c r="B10" t="s">
         <v>311</v>
       </c>
-      <c r="D10" s="28" t="s">
+      <c r="D10" s="29" t="s">
         <v>312</v>
       </c>
       <c r="E10" s="2" t="s">
@@ -5748,19 +5749,19 @@
       <c r="F10" t="s">
         <v>314</v>
       </c>
-      <c r="G10" s="25">
+      <c r="G10" s="26">
         <v>450</v>
       </c>
-      <c r="H10" s="25" t="s">
+      <c r="H10" s="26" t="s">
         <v>315</v>
       </c>
-      <c r="I10" s="12" t="s">
+      <c r="I10" s="13" t="s">
         <v>316</v>
       </c>
       <c r="J10" t="s">
         <v>285</v>
       </c>
-      <c r="K10" s="31" t="s">
+      <c r="K10" s="32" t="s">
         <v>317</v>
       </c>
       <c r="M10" s="4">
@@ -5769,13 +5770,13 @@
       <c r="N10" s="4" t="s">
         <v>209</v>
       </c>
-      <c r="O10" s="33">
+      <c r="O10" s="34">
         <v>4</v>
       </c>
-      <c r="P10" s="33" t="s">
+      <c r="P10" s="34" t="s">
         <v>227</v>
       </c>
-      <c r="Q10" s="32" t="s">
+      <c r="Q10" s="33" t="s">
         <v>310</v>
       </c>
     </row>
@@ -5790,13 +5791,13 @@
       <c r="N11" s="4" t="s">
         <v>319</v>
       </c>
-      <c r="O11" s="33">
+      <c r="O11" s="34">
         <v>5</v>
       </c>
-      <c r="P11" s="33" t="s">
+      <c r="P11" s="34" t="s">
         <v>320</v>
       </c>
-      <c r="Q11" s="32" t="s">
+      <c r="Q11" s="33" t="s">
         <v>310</v>
       </c>
     </row>
@@ -5807,10 +5808,10 @@
       <c r="B12" t="s">
         <v>321</v>
       </c>
-      <c r="C12" s="12" t="s">
+      <c r="C12" s="13" t="s">
         <v>322</v>
       </c>
-      <c r="D12" s="28" t="s">
+      <c r="D12" s="29" t="s">
         <v>323</v>
       </c>
       <c r="E12" s="2" t="s">
@@ -5819,13 +5820,13 @@
       <c r="F12" t="s">
         <v>325</v>
       </c>
-      <c r="G12" s="25">
+      <c r="G12" s="26">
         <v>450</v>
       </c>
-      <c r="H12" s="25">
+      <c r="H12" s="26">
         <v>23</v>
       </c>
-      <c r="I12" s="12" t="s">
+      <c r="I12" s="13" t="s">
         <v>326</v>
       </c>
       <c r="J12" t="s">
@@ -5834,16 +5835,16 @@
       <c r="M12" s="4">
         <v>6</v>
       </c>
-      <c r="N12" s="35" t="s">
+      <c r="N12" s="36" t="s">
         <v>286</v>
       </c>
-      <c r="O12" s="33">
+      <c r="O12" s="34">
         <v>6</v>
       </c>
-      <c r="P12" s="33" t="s">
+      <c r="P12" s="34" t="s">
         <v>327</v>
       </c>
-      <c r="Q12" s="32" t="s">
+      <c r="Q12" s="33" t="s">
         <v>310</v>
       </c>
     </row>
@@ -5854,10 +5855,10 @@
       <c r="B13" s="1" t="s">
         <v>328</v>
       </c>
-      <c r="C13" s="12" t="s">
+      <c r="C13" s="13" t="s">
         <v>329</v>
       </c>
-      <c r="D13" s="28" t="s">
+      <c r="D13" s="29" t="s">
         <v>330</v>
       </c>
       <c r="E13" s="2" t="s">
@@ -5866,13 +5867,13 @@
       <c r="F13" t="s">
         <v>332</v>
       </c>
-      <c r="G13" s="25">
+      <c r="G13" s="26">
         <v>450</v>
       </c>
-      <c r="H13" s="25">
+      <c r="H13" s="26">
         <v>28</v>
       </c>
-      <c r="I13" s="12" t="s">
+      <c r="I13" s="13" t="s">
         <v>333</v>
       </c>
       <c r="J13" t="s">
@@ -5887,13 +5888,13 @@
       <c r="N13" s="4" t="s">
         <v>219</v>
       </c>
-      <c r="O13" s="33">
+      <c r="O13" s="34">
         <v>7</v>
       </c>
-      <c r="P13" s="33" t="s">
+      <c r="P13" s="34" t="s">
         <v>249</v>
       </c>
-      <c r="Q13" s="32" t="s">
+      <c r="Q13" s="33" t="s">
         <v>310</v>
       </c>
     </row>
@@ -5904,23 +5905,23 @@
       <c r="B14" t="s">
         <v>336</v>
       </c>
-      <c r="C14" s="27">
+      <c r="C14" s="28">
         <v>0.48</v>
       </c>
-      <c r="D14" s="28" t="s">
+      <c r="D14" s="29" t="s">
         <v>337</v>
       </c>
       <c r="E14" s="2"/>
       <c r="F14" t="s">
         <v>338</v>
       </c>
-      <c r="G14" s="25">
+      <c r="G14" s="26">
         <v>450</v>
       </c>
-      <c r="H14" s="25">
+      <c r="H14" s="26">
         <v>45</v>
       </c>
-      <c r="I14" s="12" t="s">
+      <c r="I14" s="13" t="s">
         <v>339</v>
       </c>
       <c r="M14" s="4">
@@ -5929,13 +5930,13 @@
       <c r="N14" s="4" t="s">
         <v>217</v>
       </c>
-      <c r="O14" s="33">
+      <c r="O14" s="34">
         <v>8</v>
       </c>
-      <c r="P14" s="33" t="s">
+      <c r="P14" s="34" t="s">
         <v>340</v>
       </c>
-      <c r="Q14" s="32" t="s">
+      <c r="Q14" s="33" t="s">
         <v>328</v>
       </c>
     </row>
@@ -5946,7 +5947,7 @@
       <c r="B15" t="s">
         <v>286</v>
       </c>
-      <c r="C15" s="27">
+      <c r="C15" s="28">
         <v>0.4</v>
       </c>
       <c r="D15" s="2" t="s">
@@ -5965,13 +5966,13 @@
       <c r="N15" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="O15" s="33">
+      <c r="O15" s="34">
         <v>9</v>
       </c>
-      <c r="P15" s="33" t="s">
+      <c r="P15" s="34" t="s">
         <v>342</v>
       </c>
-      <c r="Q15" s="32" t="s">
+      <c r="Q15" s="33" t="s">
         <v>328</v>
       </c>
     </row>
@@ -5982,10 +5983,10 @@
       <c r="B16" s="1" t="s">
         <v>343</v>
       </c>
-      <c r="C16" s="12" t="s">
+      <c r="C16" s="13" t="s">
         <v>344</v>
       </c>
-      <c r="D16" s="28" t="s">
+      <c r="D16" s="29" t="s">
         <v>345</v>
       </c>
       <c r="E16" s="2" t="s">
@@ -5994,13 +5995,13 @@
       <c r="F16" t="s">
         <v>347</v>
       </c>
-      <c r="G16" s="25">
+      <c r="G16" s="26">
         <v>450</v>
       </c>
-      <c r="H16" s="25">
+      <c r="H16" s="26">
         <v>23</v>
       </c>
-      <c r="I16" s="12" t="s">
+      <c r="I16" s="13" t="s">
         <v>348</v>
       </c>
       <c r="K16">
@@ -6012,13 +6013,13 @@
       <c r="N16" s="4" t="s">
         <v>349</v>
       </c>
-      <c r="O16" s="33">
+      <c r="O16" s="34">
         <v>10</v>
       </c>
-      <c r="P16" s="33" t="s">
+      <c r="P16" s="34" t="s">
         <v>74</v>
       </c>
-      <c r="Q16" s="32" t="s">
+      <c r="Q16" s="33" t="s">
         <v>328</v>
       </c>
     </row>
@@ -6029,37 +6030,37 @@
       <c r="B17" t="s">
         <v>286</v>
       </c>
-      <c r="C17" s="12" t="s">
+      <c r="C17" s="13" t="s">
         <v>350</v>
       </c>
-      <c r="D17" s="28" t="s">
+      <c r="D17" s="29" t="s">
         <v>351</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>352</v>
       </c>
-      <c r="G17" s="25">
+      <c r="G17" s="26">
         <v>450</v>
       </c>
-      <c r="H17" s="25">
+      <c r="H17" s="26">
         <v>36</v>
       </c>
-      <c r="I17" s="12" t="s">
+      <c r="I17" s="13" t="s">
         <v>353</v>
       </c>
       <c r="M17" s="4">
         <v>11</v>
       </c>
-      <c r="N17" s="35" t="s">
+      <c r="N17" s="36" t="s">
         <v>354</v>
       </c>
-      <c r="O17" s="33">
+      <c r="O17" s="34">
         <v>11</v>
       </c>
-      <c r="P17" s="33" t="s">
+      <c r="P17" s="34" t="s">
         <v>355</v>
       </c>
-      <c r="Q17" s="32" t="s">
+      <c r="Q17" s="33" t="s">
         <v>356</v>
       </c>
     </row>
@@ -6070,7 +6071,7 @@
       <c r="B18" t="s">
         <v>357</v>
       </c>
-      <c r="C18" s="12" t="s">
+      <c r="C18" s="13" t="s">
         <v>358</v>
       </c>
       <c r="D18" s="2" t="s">
@@ -6086,13 +6087,13 @@
       <c r="N18" s="4" t="s">
         <v>361</v>
       </c>
-      <c r="O18" s="33">
+      <c r="O18" s="34">
         <v>12</v>
       </c>
-      <c r="P18" s="33" t="s">
+      <c r="P18" s="34" t="s">
         <v>362</v>
       </c>
-      <c r="Q18" s="32" t="s">
+      <c r="Q18" s="33" t="s">
         <v>310</v>
       </c>
     </row>
@@ -6103,7 +6104,7 @@
       <c r="B19" s="1" t="s">
         <v>363</v>
       </c>
-      <c r="C19" s="12" t="s">
+      <c r="C19" s="13" t="s">
         <v>364</v>
       </c>
       <c r="D19" s="2" t="s">
@@ -6121,27 +6122,27 @@
       <c r="B20" t="s">
         <v>367</v>
       </c>
-      <c r="C20" s="12" t="s">
+      <c r="C20" s="13" t="s">
         <v>368</v>
       </c>
-      <c r="D20" s="28" t="s">
+      <c r="D20" s="29" t="s">
         <v>369</v>
       </c>
       <c r="E20" s="2"/>
-      <c r="G20" s="25">
+      <c r="G20" s="26">
         <v>400</v>
       </c>
-      <c r="H20" s="25">
+      <c r="H20" s="26">
         <v>9</v>
       </c>
-      <c r="I20" s="12" t="s">
+      <c r="I20" s="13" t="s">
         <v>370</v>
       </c>
-      <c r="K20" s="31" t="s">
+      <c r="K20" s="32" t="s">
         <v>371</v>
       </c>
-      <c r="L20" s="32"/>
-      <c r="M20" s="36" t="s">
+      <c r="L20" s="33"/>
+      <c r="M20" s="37" t="s">
         <v>372</v>
       </c>
     </row>
@@ -6152,29 +6153,29 @@
       <c r="B21" t="s">
         <v>373</v>
       </c>
-      <c r="C21" s="12" t="s">
+      <c r="C21" s="13" t="s">
         <v>374</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>369</v>
       </c>
       <c r="E21" s="2"/>
-      <c r="G21" s="25">
+      <c r="G21" s="26">
         <v>400</v>
       </c>
-      <c r="H21" s="25">
+      <c r="H21" s="26">
         <v>30</v>
       </c>
-      <c r="I21" s="12" t="s">
+      <c r="I21" s="13" t="s">
         <v>370</v>
       </c>
-      <c r="K21" s="31" t="s">
+      <c r="K21" s="32" t="s">
         <v>371</v>
       </c>
-      <c r="L21" s="32">
+      <c r="L21" s="33">
         <v>1</v>
       </c>
-      <c r="M21" s="32" t="s">
+      <c r="M21" s="33" t="s">
         <v>375</v>
       </c>
     </row>
@@ -6185,29 +6186,29 @@
       <c r="B22" t="s">
         <v>376</v>
       </c>
-      <c r="C22" s="12" t="s">
+      <c r="C22" s="13" t="s">
         <v>377</v>
       </c>
       <c r="D22" s="2" t="s">
         <v>369</v>
       </c>
       <c r="E22" s="2"/>
-      <c r="G22" s="25">
+      <c r="G22" s="26">
         <v>400</v>
       </c>
-      <c r="H22" s="25">
+      <c r="H22" s="26">
         <v>20</v>
       </c>
-      <c r="I22" s="12" t="s">
+      <c r="I22" s="13" t="s">
         <v>370</v>
       </c>
-      <c r="K22" s="31" t="s">
+      <c r="K22" s="32" t="s">
         <v>371</v>
       </c>
-      <c r="L22" s="32">
+      <c r="L22" s="33">
         <v>2</v>
       </c>
-      <c r="M22" s="32" t="s">
+      <c r="M22" s="33" t="s">
         <v>378</v>
       </c>
     </row>
@@ -6218,26 +6219,26 @@
       <c r="B23" t="s">
         <v>379</v>
       </c>
-      <c r="C23" s="27">
+      <c r="C23" s="28">
         <v>0.29</v>
       </c>
       <c r="D23" s="2" t="s">
         <v>380</v>
       </c>
       <c r="E23" s="2"/>
-      <c r="G23" s="25">
+      <c r="G23" s="26">
         <v>400</v>
       </c>
-      <c r="H23" s="25">
+      <c r="H23" s="26">
         <v>29</v>
       </c>
-      <c r="I23" s="12" t="s">
+      <c r="I23" s="13" t="s">
         <v>370</v>
       </c>
       <c r="J23" t="s">
         <v>285</v>
       </c>
-      <c r="L23" s="32"/>
+      <c r="L23" s="33"/>
     </row>
     <row r="24" spans="1:10">
       <c r="A24">
@@ -6246,10 +6247,10 @@
       <c r="B24" t="s">
         <v>217</v>
       </c>
-      <c r="C24" s="12" t="s">
+      <c r="C24" s="13" t="s">
         <v>381</v>
       </c>
-      <c r="D24" s="28" t="s">
+      <c r="D24" s="29" t="s">
         <v>382</v>
       </c>
       <c r="E24" s="2" t="s">
@@ -6258,13 +6259,13 @@
       <c r="F24" t="s">
         <v>384</v>
       </c>
-      <c r="G24" s="25">
+      <c r="G24" s="26">
         <v>550</v>
       </c>
-      <c r="H24" s="25">
+      <c r="H24" s="26">
         <v>30</v>
       </c>
-      <c r="I24" s="12" t="s">
+      <c r="I24" s="13" t="s">
         <v>385</v>
       </c>
       <c r="J24" t="s">
@@ -6278,10 +6279,10 @@
       <c r="B25" t="s">
         <v>386</v>
       </c>
-      <c r="C25" s="12" t="s">
+      <c r="C25" s="13" t="s">
         <v>387</v>
       </c>
-      <c r="D25" s="28" t="s">
+      <c r="D25" s="29" t="s">
         <v>388</v>
       </c>
       <c r="E25" s="2" t="s">
@@ -6290,19 +6291,19 @@
       <c r="F25" t="s">
         <v>338</v>
       </c>
-      <c r="G25" s="25">
+      <c r="G25" s="26">
         <v>550</v>
       </c>
-      <c r="H25" s="11" t="s">
+      <c r="H25" s="12" t="s">
         <v>390</v>
       </c>
-      <c r="I25" s="12" t="s">
+      <c r="I25" s="13" t="s">
         <v>391</v>
       </c>
       <c r="J25" t="s">
         <v>285</v>
       </c>
-      <c r="K25" s="31" t="s">
+      <c r="K25" s="32" t="s">
         <v>392</v>
       </c>
     </row>
@@ -6313,20 +6314,20 @@
       <c r="B26" t="s">
         <v>393</v>
       </c>
-      <c r="C26" s="12" t="s">
+      <c r="C26" s="13" t="s">
         <v>394</v>
       </c>
       <c r="D26" s="2" t="s">
         <v>388</v>
       </c>
       <c r="E26" s="2"/>
-      <c r="G26" s="25">
+      <c r="G26" s="26">
         <v>550</v>
       </c>
-      <c r="H26" s="11" t="s">
+      <c r="H26" s="12" t="s">
         <v>395</v>
       </c>
-      <c r="I26" s="12" t="s">
+      <c r="I26" s="13" t="s">
         <v>391</v>
       </c>
       <c r="J26" t="s">
@@ -6340,20 +6341,20 @@
       <c r="B27" t="s">
         <v>396</v>
       </c>
-      <c r="C27" s="12" t="s">
+      <c r="C27" s="13" t="s">
         <v>397</v>
       </c>
       <c r="D27" s="2" t="s">
         <v>388</v>
       </c>
       <c r="E27" s="2"/>
-      <c r="G27" s="25">
+      <c r="G27" s="26">
         <v>550</v>
       </c>
-      <c r="H27" s="11" t="s">
+      <c r="H27" s="12" t="s">
         <v>398</v>
       </c>
-      <c r="I27" s="12" t="s">
+      <c r="I27" s="13" t="s">
         <v>391</v>
       </c>
       <c r="J27" t="s">
@@ -6367,17 +6368,17 @@
       <c r="B28" t="s">
         <v>399</v>
       </c>
-      <c r="C28" s="12" t="s">
+      <c r="C28" s="13" t="s">
         <v>400</v>
       </c>
       <c r="D28" s="2" t="s">
         <v>401</v>
       </c>
       <c r="E28" s="2"/>
-      <c r="G28" s="25">
+      <c r="G28" s="26">
         <v>400</v>
       </c>
-      <c r="H28" s="25">
+      <c r="H28" s="26">
         <v>40</v>
       </c>
     </row>
@@ -6388,7 +6389,7 @@
       <c r="B29" s="1" t="s">
         <v>310</v>
       </c>
-      <c r="C29" s="12" t="s">
+      <c r="C29" s="13" t="s">
         <v>402</v>
       </c>
       <c r="D29" s="2" t="s">
@@ -6398,19 +6399,19 @@
       <c r="F29" t="s">
         <v>404</v>
       </c>
-      <c r="G29" s="25">
+      <c r="G29" s="26">
         <v>450</v>
       </c>
-      <c r="H29" s="25">
+      <c r="H29" s="26">
         <v>47</v>
       </c>
-      <c r="I29" s="12" t="s">
+      <c r="I29" s="13" t="s">
         <v>405</v>
       </c>
       <c r="J29" t="s">
         <v>406</v>
       </c>
-      <c r="K29" s="31" t="s">
+      <c r="K29" s="32" t="s">
         <v>317</v>
       </c>
     </row>
@@ -6421,20 +6422,20 @@
       <c r="B30" t="s">
         <v>407</v>
       </c>
-      <c r="C30" s="12" t="s">
+      <c r="C30" s="13" t="s">
         <v>408</v>
       </c>
       <c r="D30" s="2" t="s">
         <v>409</v>
       </c>
       <c r="E30" s="2"/>
-      <c r="G30" s="25">
+      <c r="G30" s="26">
         <v>450</v>
       </c>
-      <c r="H30" s="25">
+      <c r="H30" s="26">
         <v>41</v>
       </c>
-      <c r="I30" s="12" t="s">
+      <c r="I30" s="13" t="s">
         <v>410</v>
       </c>
       <c r="J30" t="s">
@@ -6451,7 +6452,7 @@
       <c r="B31" t="s">
         <v>399</v>
       </c>
-      <c r="C31" s="12" t="s">
+      <c r="C31" s="13" t="s">
         <v>412</v>
       </c>
       <c r="D31" s="2" t="s">
@@ -6461,13 +6462,13 @@
       <c r="F31" t="s">
         <v>414</v>
       </c>
-      <c r="G31" s="25" t="s">
+      <c r="G31" s="26" t="s">
         <v>288</v>
       </c>
-      <c r="H31" s="25" t="s">
+      <c r="H31" s="26" t="s">
         <v>415</v>
       </c>
-      <c r="I31" s="12" t="s">
+      <c r="I31" s="13" t="s">
         <v>416</v>
       </c>
       <c r="K31" t="s">
@@ -6481,16 +6482,16 @@
       <c r="B32" t="s">
         <v>418</v>
       </c>
-      <c r="C32" s="12" t="s">
+      <c r="C32" s="13" t="s">
         <v>419</v>
       </c>
       <c r="D32" t="s">
         <v>420</v>
       </c>
-      <c r="G32" s="25">
+      <c r="G32" s="26">
         <v>450</v>
       </c>
-      <c r="I32" s="12" t="s">
+      <c r="I32" s="13" t="s">
         <v>421</v>
       </c>
     </row>
@@ -6501,7 +6502,7 @@
       <c r="B33" t="s">
         <v>422</v>
       </c>
-      <c r="C33" s="29">
+      <c r="C33" s="30">
         <v>0.249</v>
       </c>
       <c r="D33" t="s">
@@ -6555,9 +6556,9 @@
     <col min="1" max="1" width="12.7232142857143" customWidth="1"/>
     <col min="2" max="2" width="9.8125" customWidth="1"/>
     <col min="3" max="3" width="14.4553571428571" customWidth="1"/>
-    <col min="4" max="4" width="20.4553571428571" style="11" customWidth="1"/>
-    <col min="5" max="5" width="11.4553571428571" style="11" customWidth="1"/>
-    <col min="6" max="6" width="12.9107142857143" style="11" customWidth="1"/>
+    <col min="4" max="4" width="20.4553571428571" style="12" customWidth="1"/>
+    <col min="5" max="5" width="11.4553571428571" style="12" customWidth="1"/>
+    <col min="6" max="6" width="12.9107142857143" style="12" customWidth="1"/>
     <col min="7" max="7" width="17.6339285714286" customWidth="1"/>
   </cols>
   <sheetData>
@@ -6571,13 +6572,13 @@
       <c r="C1" t="s">
         <v>423</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="D1" s="13" t="s">
         <v>424</v>
       </c>
-      <c r="E1" s="12" t="s">
+      <c r="E1" s="13" t="s">
         <v>425</v>
       </c>
-      <c r="F1" s="12" t="s">
+      <c r="F1" s="13" t="s">
         <v>426</v>
       </c>
       <c r="G1" t="s">
@@ -6594,13 +6595,13 @@
       <c r="C2" s="4" t="s">
         <v>428</v>
       </c>
-      <c r="D2" s="13" t="s">
+      <c r="D2" s="14" t="s">
         <v>429</v>
       </c>
-      <c r="E2" s="13" t="s">
+      <c r="E2" s="14" t="s">
         <v>430</v>
       </c>
-      <c r="F2" s="13" t="s">
+      <c r="F2" s="14" t="s">
         <v>431</v>
       </c>
       <c r="G2" s="4" t="s">
@@ -6613,13 +6614,13 @@
       <c r="C3" s="4" t="s">
         <v>428</v>
       </c>
-      <c r="D3" s="13" t="s">
+      <c r="D3" s="14" t="s">
         <v>433</v>
       </c>
-      <c r="E3" s="13" t="s">
+      <c r="E3" s="14" t="s">
         <v>434</v>
       </c>
-      <c r="F3" s="13" t="s">
+      <c r="F3" s="14" t="s">
         <v>435</v>
       </c>
       <c r="G3" s="4" t="s">
@@ -6632,13 +6633,13 @@
       <c r="C4" s="4" t="s">
         <v>428</v>
       </c>
-      <c r="D4" s="13" t="s">
+      <c r="D4" s="14" t="s">
         <v>437</v>
       </c>
-      <c r="E4" s="13" t="s">
+      <c r="E4" s="14" t="s">
         <v>438</v>
       </c>
-      <c r="F4" s="13" t="s">
+      <c r="F4" s="14" t="s">
         <v>439</v>
       </c>
       <c r="G4" s="4" t="s">
@@ -6651,13 +6652,13 @@
       <c r="C5" s="4" t="s">
         <v>428</v>
       </c>
-      <c r="D5" s="13" t="s">
+      <c r="D5" s="14" t="s">
         <v>441</v>
       </c>
-      <c r="E5" s="13" t="s">
+      <c r="E5" s="14" t="s">
         <v>442</v>
       </c>
-      <c r="F5" s="13" t="s">
+      <c r="F5" s="14" t="s">
         <v>443</v>
       </c>
       <c r="G5" s="4" t="s">
@@ -6670,13 +6671,13 @@
       <c r="C6" s="4" t="s">
         <v>428</v>
       </c>
-      <c r="D6" s="13" t="s">
+      <c r="D6" s="14" t="s">
         <v>445</v>
       </c>
-      <c r="E6" s="13" t="s">
+      <c r="E6" s="14" t="s">
         <v>446</v>
       </c>
-      <c r="F6" s="13" t="s">
+      <c r="F6" s="14" t="s">
         <v>447</v>
       </c>
       <c r="G6" s="4" t="s">
@@ -6689,13 +6690,13 @@
       <c r="C7" s="4" t="s">
         <v>428</v>
       </c>
-      <c r="D7" s="13">
+      <c r="D7" s="14">
         <v>0</v>
       </c>
-      <c r="E7" s="13">
+      <c r="E7" s="14">
         <v>0</v>
       </c>
-      <c r="F7" s="13">
+      <c r="F7" s="14">
         <v>0</v>
       </c>
       <c r="G7" s="4" t="s">
@@ -6708,13 +6709,13 @@
       <c r="C8" s="4" t="s">
         <v>428</v>
       </c>
-      <c r="D8" s="13">
+      <c r="D8" s="14">
         <v>0</v>
       </c>
-      <c r="E8" s="13">
+      <c r="E8" s="14">
         <v>0</v>
       </c>
-      <c r="F8" s="13">
+      <c r="F8" s="14">
         <v>0</v>
       </c>
       <c r="G8" s="4" t="s">
@@ -6727,13 +6728,13 @@
       <c r="C9" s="4" t="s">
         <v>428</v>
       </c>
-      <c r="D9" s="13">
+      <c r="D9" s="14">
         <v>0</v>
       </c>
-      <c r="E9" s="13">
+      <c r="E9" s="14">
         <v>0</v>
       </c>
-      <c r="F9" s="13">
+      <c r="F9" s="14">
         <v>0</v>
       </c>
       <c r="G9" s="4" t="s">
@@ -6744,13 +6745,13 @@
       <c r="A10" s="4"/>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
-      <c r="D10" s="14" t="s">
+      <c r="D10" s="15" t="s">
         <v>452</v>
       </c>
-      <c r="E10" s="14" t="s">
+      <c r="E10" s="15" t="s">
         <v>453</v>
       </c>
-      <c r="F10" s="14" t="s">
+      <c r="F10" s="15" t="s">
         <v>454</v>
       </c>
       <c r="G10" s="3" t="s">
@@ -6763,13 +6764,13 @@
       <c r="C11" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="D11" s="13" t="s">
+      <c r="D11" s="14" t="s">
         <v>456</v>
       </c>
-      <c r="E11" s="13" t="s">
+      <c r="E11" s="14" t="s">
         <v>457</v>
       </c>
-      <c r="F11" s="13" t="s">
+      <c r="F11" s="14" t="s">
         <v>458</v>
       </c>
       <c r="G11" s="4" t="s">
@@ -6782,13 +6783,13 @@
       <c r="C12" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="D12" s="15">
+      <c r="D12" s="16">
         <v>1029</v>
       </c>
-      <c r="E12" s="13" t="s">
+      <c r="E12" s="14" t="s">
         <v>459</v>
       </c>
-      <c r="F12" s="13" t="s">
+      <c r="F12" s="14" t="s">
         <v>460</v>
       </c>
       <c r="G12" s="4" t="s">
@@ -6801,13 +6802,13 @@
       <c r="C13" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="D13" s="13" t="s">
+      <c r="D13" s="14" t="s">
         <v>461</v>
       </c>
-      <c r="E13" s="13" t="s">
+      <c r="E13" s="14" t="s">
         <v>462</v>
       </c>
-      <c r="F13" s="13" t="s">
+      <c r="F13" s="14" t="s">
         <v>463</v>
       </c>
       <c r="G13" s="4" t="s">
@@ -6820,13 +6821,13 @@
       <c r="C14" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="D14" s="13" t="s">
+      <c r="D14" s="14" t="s">
         <v>464</v>
       </c>
-      <c r="E14" s="13" t="s">
+      <c r="E14" s="14" t="s">
         <v>438</v>
       </c>
-      <c r="F14" s="13" t="s">
+      <c r="F14" s="14" t="s">
         <v>465</v>
       </c>
       <c r="G14" s="4" t="s">
@@ -6839,13 +6840,13 @@
       <c r="C15" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="D15" s="13" t="s">
+      <c r="D15" s="14" t="s">
         <v>466</v>
       </c>
-      <c r="E15" s="13" t="s">
+      <c r="E15" s="14" t="s">
         <v>467</v>
       </c>
-      <c r="F15" s="13" t="s">
+      <c r="F15" s="14" t="s">
         <v>468</v>
       </c>
       <c r="G15" s="4" t="s">
@@ -6858,13 +6859,13 @@
       <c r="C16" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="D16" s="13">
+      <c r="D16" s="14">
         <v>0</v>
       </c>
-      <c r="E16" s="13">
+      <c r="E16" s="14">
         <v>0</v>
       </c>
-      <c r="F16" s="13">
+      <c r="F16" s="14">
         <v>0</v>
       </c>
       <c r="G16" s="4" t="s">
@@ -6877,13 +6878,13 @@
       <c r="C17" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="D17" s="13">
+      <c r="D17" s="14">
         <v>0</v>
       </c>
-      <c r="E17" s="13">
+      <c r="E17" s="14">
         <v>0</v>
       </c>
-      <c r="F17" s="13">
+      <c r="F17" s="14">
         <v>0</v>
       </c>
       <c r="G17" s="4" t="s">
@@ -6896,13 +6897,13 @@
       <c r="C18" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="D18" s="13">
+      <c r="D18" s="14">
         <v>0</v>
       </c>
-      <c r="E18" s="13">
+      <c r="E18" s="14">
         <v>0</v>
       </c>
-      <c r="F18" s="13">
+      <c r="F18" s="14">
         <v>0</v>
       </c>
       <c r="G18" s="4" t="s">
@@ -6913,13 +6914,13 @@
       <c r="A19" s="4"/>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
-      <c r="D19" s="14" t="s">
+      <c r="D19" s="15" t="s">
         <v>469</v>
       </c>
-      <c r="E19" s="14" t="s">
+      <c r="E19" s="15" t="s">
         <v>470</v>
       </c>
-      <c r="F19" s="14" t="s">
+      <c r="F19" s="15" t="s">
         <v>471</v>
       </c>
       <c r="G19" s="3" t="s">
@@ -6927,513 +6928,513 @@
       </c>
     </row>
     <row r="20" spans="1:7">
-      <c r="A20" s="16" t="s">
+      <c r="A20" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="B20" s="16" t="s">
+      <c r="B20" s="17" t="s">
         <v>472</v>
       </c>
-      <c r="C20" s="16" t="s">
+      <c r="C20" s="17" t="s">
         <v>428</v>
       </c>
-      <c r="D20" s="17" t="s">
+      <c r="D20" s="18" t="s">
         <v>473</v>
       </c>
-      <c r="E20" s="17" t="s">
+      <c r="E20" s="18" t="s">
         <v>474</v>
       </c>
-      <c r="F20" s="17" t="s">
+      <c r="F20" s="18" t="s">
         <v>475</v>
       </c>
-      <c r="G20" s="16" t="s">
+      <c r="G20" s="17" t="s">
         <v>432</v>
       </c>
     </row>
     <row r="21" spans="1:7">
-      <c r="A21" s="16"/>
-      <c r="B21" s="16"/>
-      <c r="C21" s="16" t="s">
+      <c r="A21" s="17"/>
+      <c r="B21" s="17"/>
+      <c r="C21" s="17" t="s">
         <v>428</v>
       </c>
-      <c r="D21" s="17" t="s">
+      <c r="D21" s="18" t="s">
         <v>476</v>
       </c>
-      <c r="E21" s="17" t="s">
+      <c r="E21" s="18" t="s">
         <v>477</v>
       </c>
-      <c r="F21" s="17" t="s">
+      <c r="F21" s="18" t="s">
         <v>478</v>
       </c>
-      <c r="G21" s="16" t="s">
+      <c r="G21" s="17" t="s">
         <v>436</v>
       </c>
     </row>
     <row r="22" spans="1:7">
-      <c r="A22" s="16"/>
-      <c r="B22" s="16"/>
-      <c r="C22" s="16" t="s">
+      <c r="A22" s="17"/>
+      <c r="B22" s="17"/>
+      <c r="C22" s="17" t="s">
         <v>428</v>
       </c>
-      <c r="D22" s="17" t="s">
+      <c r="D22" s="18" t="s">
         <v>479</v>
       </c>
-      <c r="E22" s="17" t="s">
+      <c r="E22" s="18" t="s">
         <v>480</v>
       </c>
-      <c r="F22" s="17" t="s">
+      <c r="F22" s="18" t="s">
         <v>481</v>
       </c>
-      <c r="G22" s="16" t="s">
+      <c r="G22" s="17" t="s">
         <v>440</v>
       </c>
     </row>
     <row r="23" spans="1:7">
-      <c r="A23" s="16"/>
-      <c r="B23" s="16"/>
-      <c r="C23" s="16" t="s">
+      <c r="A23" s="17"/>
+      <c r="B23" s="17"/>
+      <c r="C23" s="17" t="s">
         <v>428</v>
       </c>
-      <c r="D23" s="17" t="s">
+      <c r="D23" s="18" t="s">
         <v>482</v>
       </c>
-      <c r="E23" s="17" t="s">
+      <c r="E23" s="18" t="s">
         <v>483</v>
       </c>
-      <c r="F23" s="17" t="s">
+      <c r="F23" s="18" t="s">
         <v>484</v>
       </c>
-      <c r="G23" s="16" t="s">
+      <c r="G23" s="17" t="s">
         <v>444</v>
       </c>
     </row>
     <row r="24" spans="1:7">
-      <c r="A24" s="16"/>
-      <c r="B24" s="16"/>
-      <c r="C24" s="16" t="s">
+      <c r="A24" s="17"/>
+      <c r="B24" s="17"/>
+      <c r="C24" s="17" t="s">
         <v>428</v>
       </c>
-      <c r="D24" s="17" t="s">
+      <c r="D24" s="18" t="s">
         <v>485</v>
       </c>
-      <c r="E24" s="17" t="s">
+      <c r="E24" s="18" t="s">
         <v>486</v>
       </c>
-      <c r="F24" s="17" t="s">
+      <c r="F24" s="18" t="s">
         <v>487</v>
       </c>
-      <c r="G24" s="16" t="s">
+      <c r="G24" s="17" t="s">
         <v>448</v>
       </c>
     </row>
     <row r="25" spans="1:7">
-      <c r="A25" s="16"/>
-      <c r="B25" s="16"/>
-      <c r="C25" s="16" t="s">
+      <c r="A25" s="17"/>
+      <c r="B25" s="17"/>
+      <c r="C25" s="17" t="s">
         <v>428</v>
       </c>
-      <c r="D25" s="17" t="s">
+      <c r="D25" s="18" t="s">
         <v>488</v>
       </c>
-      <c r="E25" s="17" t="s">
+      <c r="E25" s="18" t="s">
         <v>489</v>
       </c>
-      <c r="F25" s="17" t="s">
+      <c r="F25" s="18" t="s">
         <v>490</v>
       </c>
-      <c r="G25" s="16" t="s">
+      <c r="G25" s="17" t="s">
         <v>449</v>
       </c>
     </row>
     <row r="26" spans="1:7">
-      <c r="A26" s="16"/>
-      <c r="B26" s="16"/>
-      <c r="C26" s="16" t="s">
+      <c r="A26" s="17"/>
+      <c r="B26" s="17"/>
+      <c r="C26" s="17" t="s">
         <v>428</v>
       </c>
-      <c r="D26" s="17" t="s">
+      <c r="D26" s="18" t="s">
         <v>488</v>
       </c>
-      <c r="E26" s="17" t="s">
+      <c r="E26" s="18" t="s">
         <v>489</v>
       </c>
-      <c r="F26" s="17" t="s">
+      <c r="F26" s="18" t="s">
         <v>491</v>
       </c>
-      <c r="G26" s="16" t="s">
+      <c r="G26" s="17" t="s">
         <v>450</v>
       </c>
     </row>
     <row r="27" spans="1:7">
-      <c r="A27" s="16"/>
-      <c r="B27" s="16"/>
-      <c r="C27" s="16" t="s">
+      <c r="A27" s="17"/>
+      <c r="B27" s="17"/>
+      <c r="C27" s="17" t="s">
         <v>428</v>
       </c>
-      <c r="D27" s="17" t="s">
+      <c r="D27" s="18" t="s">
         <v>492</v>
       </c>
-      <c r="E27" s="17" t="s">
+      <c r="E27" s="18" t="s">
         <v>493</v>
       </c>
-      <c r="F27" s="17" t="s">
+      <c r="F27" s="18" t="s">
         <v>494</v>
       </c>
-      <c r="G27" s="16" t="s">
+      <c r="G27" s="17" t="s">
         <v>451</v>
       </c>
     </row>
     <row r="28" spans="1:7">
-      <c r="A28" s="16"/>
-      <c r="B28" s="16"/>
-      <c r="C28" s="16"/>
-      <c r="D28" s="18" t="s">
+      <c r="A28" s="17"/>
+      <c r="B28" s="17"/>
+      <c r="C28" s="17"/>
+      <c r="D28" s="19" t="s">
         <v>495</v>
       </c>
-      <c r="E28" s="18" t="s">
+      <c r="E28" s="19" t="s">
         <v>496</v>
       </c>
-      <c r="F28" s="18" t="s">
+      <c r="F28" s="19" t="s">
         <v>497</v>
       </c>
-      <c r="G28" s="21" t="s">
+      <c r="G28" s="22" t="s">
         <v>455</v>
       </c>
     </row>
     <row r="29" spans="1:7">
-      <c r="A29" s="16"/>
-      <c r="B29" s="16"/>
-      <c r="C29" s="16" t="s">
+      <c r="A29" s="17"/>
+      <c r="B29" s="17"/>
+      <c r="C29" s="17" t="s">
         <v>498</v>
       </c>
-      <c r="D29" s="17" t="s">
+      <c r="D29" s="18" t="s">
         <v>499</v>
       </c>
-      <c r="E29" s="17" t="s">
+      <c r="E29" s="18" t="s">
         <v>500</v>
       </c>
-      <c r="F29" s="17" t="s">
+      <c r="F29" s="18" t="s">
         <v>501</v>
       </c>
-      <c r="G29" s="16" t="s">
+      <c r="G29" s="17" t="s">
         <v>432</v>
       </c>
     </row>
     <row r="30" spans="1:7">
-      <c r="A30" s="16"/>
-      <c r="B30" s="16"/>
-      <c r="C30" s="16" t="s">
+      <c r="A30" s="17"/>
+      <c r="B30" s="17"/>
+      <c r="C30" s="17" t="s">
         <v>498</v>
       </c>
-      <c r="D30" s="17" t="s">
+      <c r="D30" s="18" t="s">
         <v>502</v>
       </c>
-      <c r="E30" s="17" t="s">
+      <c r="E30" s="18" t="s">
         <v>503</v>
       </c>
-      <c r="F30" s="17" t="s">
+      <c r="F30" s="18" t="s">
         <v>504</v>
       </c>
-      <c r="G30" s="16" t="s">
+      <c r="G30" s="17" t="s">
         <v>436</v>
       </c>
     </row>
     <row r="31" spans="1:7">
-      <c r="A31" s="16"/>
-      <c r="B31" s="16"/>
-      <c r="C31" s="16" t="s">
+      <c r="A31" s="17"/>
+      <c r="B31" s="17"/>
+      <c r="C31" s="17" t="s">
         <v>498</v>
       </c>
-      <c r="D31" s="17" t="s">
+      <c r="D31" s="18" t="s">
         <v>479</v>
       </c>
-      <c r="E31" s="17" t="s">
+      <c r="E31" s="18" t="s">
         <v>505</v>
       </c>
-      <c r="F31" s="17" t="s">
+      <c r="F31" s="18" t="s">
         <v>506</v>
       </c>
-      <c r="G31" s="16" t="s">
+      <c r="G31" s="17" t="s">
         <v>440</v>
       </c>
     </row>
     <row r="32" spans="1:7">
-      <c r="A32" s="16"/>
-      <c r="B32" s="16"/>
-      <c r="C32" s="16" t="s">
+      <c r="A32" s="17"/>
+      <c r="B32" s="17"/>
+      <c r="C32" s="17" t="s">
         <v>498</v>
       </c>
-      <c r="D32" s="17" t="s">
+      <c r="D32" s="18" t="s">
         <v>482</v>
       </c>
-      <c r="E32" s="17" t="s">
+      <c r="E32" s="18" t="s">
         <v>462</v>
       </c>
-      <c r="F32" s="17" t="s">
+      <c r="F32" s="18" t="s">
         <v>507</v>
       </c>
-      <c r="G32" s="16" t="s">
+      <c r="G32" s="17" t="s">
         <v>444</v>
       </c>
     </row>
     <row r="33" spans="1:7">
-      <c r="A33" s="16"/>
-      <c r="B33" s="16"/>
-      <c r="C33" s="16" t="s">
+      <c r="A33" s="17"/>
+      <c r="B33" s="17"/>
+      <c r="C33" s="17" t="s">
         <v>498</v>
       </c>
-      <c r="D33" s="17" t="s">
+      <c r="D33" s="18" t="s">
         <v>508</v>
       </c>
-      <c r="E33" s="17" t="s">
+      <c r="E33" s="18" t="s">
         <v>509</v>
       </c>
-      <c r="F33" s="17" t="s">
+      <c r="F33" s="18" t="s">
         <v>510</v>
       </c>
-      <c r="G33" s="16" t="s">
+      <c r="G33" s="17" t="s">
         <v>448</v>
       </c>
     </row>
     <row r="34" spans="1:7">
-      <c r="A34" s="16"/>
-      <c r="B34" s="16"/>
-      <c r="C34" s="16" t="s">
+      <c r="A34" s="17"/>
+      <c r="B34" s="17"/>
+      <c r="C34" s="17" t="s">
         <v>498</v>
       </c>
-      <c r="D34" s="17" t="s">
+      <c r="D34" s="18" t="s">
         <v>509</v>
       </c>
-      <c r="E34" s="17" t="s">
+      <c r="E34" s="18" t="s">
         <v>462</v>
       </c>
-      <c r="F34" s="17" t="s">
+      <c r="F34" s="18" t="s">
         <v>511</v>
       </c>
-      <c r="G34" s="16" t="s">
+      <c r="G34" s="17" t="s">
         <v>449</v>
       </c>
     </row>
     <row r="35" spans="1:7">
-      <c r="A35" s="16"/>
-      <c r="B35" s="16"/>
-      <c r="C35" s="16" t="s">
+      <c r="A35" s="17"/>
+      <c r="B35" s="17"/>
+      <c r="C35" s="17" t="s">
         <v>498</v>
       </c>
-      <c r="D35" s="17" t="s">
+      <c r="D35" s="18" t="s">
         <v>509</v>
       </c>
-      <c r="E35" s="17" t="s">
+      <c r="E35" s="18" t="s">
         <v>462</v>
       </c>
-      <c r="F35" s="17" t="s">
+      <c r="F35" s="18" t="s">
         <v>511</v>
       </c>
-      <c r="G35" s="16" t="s">
+      <c r="G35" s="17" t="s">
         <v>450</v>
       </c>
     </row>
     <row r="36" spans="1:7">
-      <c r="A36" s="16"/>
-      <c r="B36" s="16"/>
-      <c r="C36" s="16" t="s">
+      <c r="A36" s="17"/>
+      <c r="B36" s="17"/>
+      <c r="C36" s="17" t="s">
         <v>498</v>
       </c>
-      <c r="D36" s="17" t="s">
+      <c r="D36" s="18" t="s">
         <v>506</v>
       </c>
-      <c r="E36" s="17" t="s">
+      <c r="E36" s="18" t="s">
         <v>462</v>
       </c>
-      <c r="F36" s="17" t="s">
+      <c r="F36" s="18" t="s">
         <v>512</v>
       </c>
-      <c r="G36" s="16" t="s">
+      <c r="G36" s="17" t="s">
         <v>451</v>
       </c>
     </row>
     <row r="37" spans="1:7">
-      <c r="A37" s="16"/>
-      <c r="B37" s="16"/>
-      <c r="C37" s="16"/>
-      <c r="D37" s="17" t="s">
+      <c r="A37" s="17"/>
+      <c r="B37" s="17"/>
+      <c r="C37" s="17"/>
+      <c r="D37" s="18" t="s">
         <v>513</v>
       </c>
-      <c r="E37" s="17" t="s">
+      <c r="E37" s="18" t="s">
         <v>514</v>
       </c>
-      <c r="F37" s="17" t="s">
+      <c r="F37" s="18" t="s">
         <v>515</v>
       </c>
-      <c r="G37" s="16" t="s">
+      <c r="G37" s="17" t="s">
         <v>455</v>
       </c>
     </row>
     <row r="38" spans="1:7">
-      <c r="A38" s="16"/>
-      <c r="B38" s="16"/>
-      <c r="C38" s="16" t="s">
+      <c r="A38" s="17"/>
+      <c r="B38" s="17"/>
+      <c r="C38" s="17" t="s">
         <v>516</v>
       </c>
-      <c r="D38" s="17" t="s">
+      <c r="D38" s="18" t="s">
         <v>517</v>
       </c>
-      <c r="E38" s="17" t="s">
+      <c r="E38" s="18" t="s">
         <v>518</v>
       </c>
-      <c r="F38" s="17" t="s">
+      <c r="F38" s="18" t="s">
         <v>519</v>
       </c>
-      <c r="G38" s="16" t="s">
+      <c r="G38" s="17" t="s">
         <v>432</v>
       </c>
     </row>
     <row r="39" spans="1:7">
-      <c r="A39" s="16"/>
-      <c r="B39" s="16"/>
-      <c r="C39" s="16" t="s">
+      <c r="A39" s="17"/>
+      <c r="B39" s="17"/>
+      <c r="C39" s="17" t="s">
         <v>516</v>
       </c>
-      <c r="D39" s="17" t="s">
+      <c r="D39" s="18" t="s">
         <v>520</v>
       </c>
-      <c r="E39" s="17" t="s">
+      <c r="E39" s="18" t="s">
         <v>518</v>
       </c>
-      <c r="F39" s="17" t="s">
+      <c r="F39" s="18" t="s">
         <v>521</v>
       </c>
-      <c r="G39" s="16" t="s">
+      <c r="G39" s="17" t="s">
         <v>436</v>
       </c>
     </row>
     <row r="40" spans="1:7">
-      <c r="A40" s="16"/>
-      <c r="B40" s="16"/>
-      <c r="C40" s="16" t="s">
+      <c r="A40" s="17"/>
+      <c r="B40" s="17"/>
+      <c r="C40" s="17" t="s">
         <v>516</v>
       </c>
-      <c r="D40" s="17" t="s">
+      <c r="D40" s="18" t="s">
         <v>462</v>
       </c>
-      <c r="E40" s="17" t="s">
+      <c r="E40" s="18" t="s">
         <v>518</v>
       </c>
-      <c r="F40" s="17" t="s">
+      <c r="F40" s="18" t="s">
         <v>509</v>
       </c>
-      <c r="G40" s="16" t="s">
+      <c r="G40" s="17" t="s">
         <v>440</v>
       </c>
     </row>
     <row r="41" spans="1:7">
-      <c r="A41" s="16"/>
-      <c r="B41" s="16"/>
-      <c r="C41" s="16" t="s">
+      <c r="A41" s="17"/>
+      <c r="B41" s="17"/>
+      <c r="C41" s="17" t="s">
         <v>516</v>
       </c>
-      <c r="D41" s="17" t="s">
+      <c r="D41" s="18" t="s">
         <v>482</v>
       </c>
-      <c r="E41" s="17" t="s">
+      <c r="E41" s="18" t="s">
         <v>518</v>
       </c>
-      <c r="F41" s="17" t="s">
+      <c r="F41" s="18" t="s">
         <v>522</v>
       </c>
-      <c r="G41" s="16" t="s">
+      <c r="G41" s="17" t="s">
         <v>444</v>
       </c>
     </row>
     <row r="42" spans="1:7">
-      <c r="A42" s="16"/>
-      <c r="B42" s="16"/>
-      <c r="C42" s="16" t="s">
+      <c r="A42" s="17"/>
+      <c r="B42" s="17"/>
+      <c r="C42" s="17" t="s">
         <v>516</v>
       </c>
-      <c r="D42" s="17" t="s">
+      <c r="D42" s="18" t="s">
         <v>485</v>
       </c>
-      <c r="E42" s="17" t="s">
+      <c r="E42" s="18" t="s">
         <v>518</v>
       </c>
-      <c r="F42" s="17" t="s">
+      <c r="F42" s="18" t="s">
         <v>467</v>
       </c>
-      <c r="G42" s="16" t="s">
+      <c r="G42" s="17" t="s">
         <v>448</v>
       </c>
     </row>
     <row r="43" spans="1:7">
-      <c r="A43" s="16"/>
-      <c r="B43" s="16"/>
-      <c r="C43" s="16" t="s">
+      <c r="A43" s="17"/>
+      <c r="B43" s="17"/>
+      <c r="C43" s="17" t="s">
         <v>516</v>
       </c>
-      <c r="D43" s="17" t="s">
+      <c r="D43" s="18" t="s">
         <v>506</v>
       </c>
-      <c r="E43" s="17" t="s">
+      <c r="E43" s="18" t="s">
         <v>518</v>
       </c>
-      <c r="F43" s="17" t="s">
+      <c r="F43" s="18" t="s">
         <v>507</v>
       </c>
-      <c r="G43" s="16" t="s">
+      <c r="G43" s="17" t="s">
         <v>449</v>
       </c>
     </row>
     <row r="44" spans="1:7">
-      <c r="A44" s="16"/>
-      <c r="B44" s="16"/>
-      <c r="C44" s="16" t="s">
+      <c r="A44" s="17"/>
+      <c r="B44" s="17"/>
+      <c r="C44" s="17" t="s">
         <v>516</v>
       </c>
-      <c r="D44" s="17" t="s">
+      <c r="D44" s="18" t="s">
         <v>509</v>
       </c>
-      <c r="E44" s="17" t="s">
+      <c r="E44" s="18" t="s">
         <v>518</v>
       </c>
-      <c r="F44" s="17" t="s">
+      <c r="F44" s="18" t="s">
         <v>507</v>
       </c>
-      <c r="G44" s="16" t="s">
+      <c r="G44" s="17" t="s">
         <v>450</v>
       </c>
     </row>
     <row r="45" spans="1:7">
-      <c r="A45" s="16"/>
-      <c r="B45" s="16"/>
-      <c r="C45" s="16" t="s">
+      <c r="A45" s="17"/>
+      <c r="B45" s="17"/>
+      <c r="C45" s="17" t="s">
         <v>516</v>
       </c>
-      <c r="D45" s="17" t="s">
+      <c r="D45" s="18" t="s">
         <v>523</v>
       </c>
-      <c r="E45" s="17" t="s">
+      <c r="E45" s="18" t="s">
         <v>518</v>
       </c>
-      <c r="F45" s="17" t="s">
+      <c r="F45" s="18" t="s">
         <v>511</v>
       </c>
-      <c r="G45" s="16" t="s">
+      <c r="G45" s="17" t="s">
         <v>451</v>
       </c>
     </row>
     <row r="46" spans="1:7">
-      <c r="A46" s="16"/>
-      <c r="B46" s="16"/>
-      <c r="C46" s="16"/>
-      <c r="D46" s="18" t="s">
+      <c r="A46" s="17"/>
+      <c r="B46" s="17"/>
+      <c r="C46" s="17"/>
+      <c r="D46" s="19" t="s">
         <v>524</v>
       </c>
-      <c r="E46" s="18" t="s">
+      <c r="E46" s="19" t="s">
         <v>518</v>
       </c>
-      <c r="F46" s="18" t="s">
+      <c r="F46" s="19" t="s">
         <v>525</v>
       </c>
-      <c r="G46" s="21" t="s">
+      <c r="G46" s="22" t="s">
         <v>455</v>
       </c>
     </row>
@@ -7447,13 +7448,13 @@
       <c r="C47" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D47" s="19" t="s">
+      <c r="D47" s="20" t="s">
         <v>526</v>
       </c>
-      <c r="E47" s="19" t="s">
+      <c r="E47" s="20" t="s">
         <v>479</v>
       </c>
-      <c r="F47" s="19" t="s">
+      <c r="F47" s="20" t="s">
         <v>527</v>
       </c>
       <c r="G47" s="5" t="s">
@@ -7466,13 +7467,13 @@
       <c r="C48" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D48" s="19" t="s">
+      <c r="D48" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="E48" s="19" t="s">
+      <c r="E48" s="20" t="s">
         <v>528</v>
       </c>
-      <c r="F48" s="19" t="s">
+      <c r="F48" s="20" t="s">
         <v>529</v>
       </c>
       <c r="G48" s="5" t="s">
@@ -7485,13 +7486,13 @@
       <c r="C49" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D49" s="19" t="s">
+      <c r="D49" s="20" t="s">
         <v>530</v>
       </c>
-      <c r="E49" s="19" t="s">
+      <c r="E49" s="20" t="s">
         <v>479</v>
       </c>
-      <c r="F49" s="19" t="s">
+      <c r="F49" s="20" t="s">
         <v>531</v>
       </c>
       <c r="G49" s="5" t="s">
@@ -7504,13 +7505,13 @@
       <c r="C50" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D50" s="19" t="s">
+      <c r="D50" s="20" t="s">
         <v>532</v>
       </c>
-      <c r="E50" s="19" t="s">
+      <c r="E50" s="20" t="s">
         <v>462</v>
       </c>
-      <c r="F50" s="19" t="s">
+      <c r="F50" s="20" t="s">
         <v>499</v>
       </c>
       <c r="G50" s="5" t="s">
@@ -7523,13 +7524,13 @@
       <c r="C51" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D51" s="19" t="s">
+      <c r="D51" s="20" t="s">
         <v>533</v>
       </c>
-      <c r="E51" s="19" t="s">
+      <c r="E51" s="20" t="s">
         <v>512</v>
       </c>
-      <c r="F51" s="19" t="s">
+      <c r="F51" s="20" t="s">
         <v>534</v>
       </c>
       <c r="G51" s="5" t="s">
@@ -7542,13 +7543,13 @@
       <c r="C52" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D52" s="19" t="s">
+      <c r="D52" s="20" t="s">
         <v>535</v>
       </c>
-      <c r="E52" s="19" t="s">
+      <c r="E52" s="20" t="s">
         <v>523</v>
       </c>
-      <c r="F52" s="19" t="s">
+      <c r="F52" s="20" t="s">
         <v>536</v>
       </c>
       <c r="G52" s="5" t="s">
@@ -7561,13 +7562,13 @@
       <c r="C53" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D53" s="19" t="s">
+      <c r="D53" s="20" t="s">
         <v>537</v>
       </c>
-      <c r="E53" s="19" t="s">
+      <c r="E53" s="20" t="s">
         <v>506</v>
       </c>
-      <c r="F53" s="19" t="s">
+      <c r="F53" s="20" t="s">
         <v>538</v>
       </c>
       <c r="G53" s="5" t="s">
@@ -7580,13 +7581,13 @@
       <c r="C54" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D54" s="19" t="s">
+      <c r="D54" s="20" t="s">
         <v>539</v>
       </c>
-      <c r="E54" s="19" t="s">
+      <c r="E54" s="20" t="s">
         <v>528</v>
       </c>
-      <c r="F54" s="19" t="s">
+      <c r="F54" s="20" t="s">
         <v>540</v>
       </c>
       <c r="G54" s="5" t="s">
@@ -7597,16 +7598,16 @@
       <c r="A55" s="5"/>
       <c r="B55" s="5"/>
       <c r="C55" s="5"/>
-      <c r="D55" s="20" t="s">
+      <c r="D55" s="21" t="s">
         <v>541</v>
       </c>
-      <c r="E55" s="20" t="s">
+      <c r="E55" s="21" t="s">
         <v>542</v>
       </c>
-      <c r="F55" s="22">
+      <c r="F55" s="23">
         <v>1469</v>
       </c>
-      <c r="G55" s="23" t="s">
+      <c r="G55" s="24" t="s">
         <v>455</v>
       </c>
     </row>
@@ -7616,13 +7617,13 @@
       <c r="C56" s="5" t="s">
         <v>543</v>
       </c>
-      <c r="D56" s="19" t="s">
+      <c r="D56" s="20" t="s">
         <v>508</v>
       </c>
-      <c r="E56" s="19" t="s">
+      <c r="E56" s="20" t="s">
         <v>479</v>
       </c>
-      <c r="F56" s="19" t="s">
+      <c r="F56" s="20" t="s">
         <v>544</v>
       </c>
       <c r="G56" s="5" t="s">
@@ -7635,13 +7636,13 @@
       <c r="C57" s="5" t="s">
         <v>543</v>
       </c>
-      <c r="D57" s="19" t="s">
+      <c r="D57" s="20" t="s">
         <v>545</v>
       </c>
-      <c r="E57" s="19" t="s">
+      <c r="E57" s="20" t="s">
         <v>528</v>
       </c>
-      <c r="F57" s="19" t="s">
+      <c r="F57" s="20" t="s">
         <v>546</v>
       </c>
       <c r="G57" s="5" t="s">
@@ -7654,13 +7655,13 @@
       <c r="C58" s="5" t="s">
         <v>543</v>
       </c>
-      <c r="D58" s="19" t="s">
+      <c r="D58" s="20" t="s">
         <v>461</v>
       </c>
-      <c r="E58" s="19" t="s">
+      <c r="E58" s="20" t="s">
         <v>479</v>
       </c>
-      <c r="F58" s="19" t="s">
+      <c r="F58" s="20" t="s">
         <v>547</v>
       </c>
       <c r="G58" s="5" t="s">
@@ -7673,13 +7674,13 @@
       <c r="C59" s="5" t="s">
         <v>543</v>
       </c>
-      <c r="D59" s="19" t="s">
+      <c r="D59" s="20" t="s">
         <v>511</v>
       </c>
-      <c r="E59" s="19" t="s">
+      <c r="E59" s="20" t="s">
         <v>462</v>
       </c>
-      <c r="F59" s="19" t="s">
+      <c r="F59" s="20" t="s">
         <v>438</v>
       </c>
       <c r="G59" s="5" t="s">
@@ -7692,13 +7693,13 @@
       <c r="C60" s="5" t="s">
         <v>543</v>
       </c>
-      <c r="D60" s="19" t="s">
+      <c r="D60" s="20" t="s">
         <v>548</v>
       </c>
-      <c r="E60" s="19" t="s">
+      <c r="E60" s="20" t="s">
         <v>549</v>
       </c>
-      <c r="F60" s="19" t="s">
+      <c r="F60" s="20" t="s">
         <v>550</v>
       </c>
       <c r="G60" s="5" t="s">
@@ -7711,13 +7712,13 @@
       <c r="C61" s="5" t="s">
         <v>543</v>
       </c>
-      <c r="D61" s="19" t="s">
+      <c r="D61" s="20" t="s">
         <v>551</v>
       </c>
-      <c r="E61" s="19" t="s">
+      <c r="E61" s="20" t="s">
         <v>523</v>
       </c>
-      <c r="F61" s="19" t="s">
+      <c r="F61" s="20" t="s">
         <v>467</v>
       </c>
       <c r="G61" s="5" t="s">
@@ -7730,13 +7731,13 @@
       <c r="C62" s="5" t="s">
         <v>543</v>
       </c>
-      <c r="D62" s="19" t="s">
+      <c r="D62" s="20" t="s">
         <v>532</v>
       </c>
-      <c r="E62" s="19" t="s">
+      <c r="E62" s="20" t="s">
         <v>506</v>
       </c>
-      <c r="F62" s="19" t="s">
+      <c r="F62" s="20" t="s">
         <v>552</v>
       </c>
       <c r="G62" s="5" t="s">
@@ -7749,13 +7750,13 @@
       <c r="C63" s="5" t="s">
         <v>543</v>
       </c>
-      <c r="D63" s="19" t="s">
+      <c r="D63" s="20" t="s">
         <v>552</v>
       </c>
-      <c r="E63" s="19" t="s">
+      <c r="E63" s="20" t="s">
         <v>512</v>
       </c>
-      <c r="F63" s="19" t="s">
+      <c r="F63" s="20" t="s">
         <v>553</v>
       </c>
       <c r="G63" s="5" t="s">
@@ -7766,16 +7767,16 @@
       <c r="A64" s="5"/>
       <c r="B64" s="5"/>
       <c r="C64" s="5"/>
-      <c r="D64" s="20" t="s">
+      <c r="D64" s="21" t="s">
         <v>554</v>
       </c>
-      <c r="E64" s="20" t="s">
+      <c r="E64" s="21" t="s">
         <v>526</v>
       </c>
-      <c r="F64" s="20" t="s">
+      <c r="F64" s="21" t="s">
         <v>555</v>
       </c>
-      <c r="G64" s="23" t="s">
+      <c r="G64" s="24" t="s">
         <v>455</v>
       </c>
     </row>
@@ -7785,13 +7786,13 @@
       <c r="C65" s="5" t="s">
         <v>556</v>
       </c>
-      <c r="D65" s="19" t="s">
+      <c r="D65" s="20" t="s">
         <v>547</v>
       </c>
-      <c r="E65" s="19" t="s">
+      <c r="E65" s="20" t="s">
         <v>522</v>
       </c>
-      <c r="F65" s="19" t="s">
+      <c r="F65" s="20" t="s">
         <v>510</v>
       </c>
       <c r="G65" s="5" t="s">
@@ -7804,13 +7805,13 @@
       <c r="C66" s="5" t="s">
         <v>556</v>
       </c>
-      <c r="D66" s="19" t="s">
+      <c r="D66" s="20" t="s">
         <v>557</v>
       </c>
-      <c r="E66" s="19" t="s">
+      <c r="E66" s="20" t="s">
         <v>467</v>
       </c>
-      <c r="F66" s="19" t="s">
+      <c r="F66" s="20" t="s">
         <v>558</v>
       </c>
       <c r="G66" s="5" t="s">
@@ -7823,13 +7824,13 @@
       <c r="C67" s="5" t="s">
         <v>556</v>
       </c>
-      <c r="D67" s="19" t="s">
+      <c r="D67" s="20" t="s">
         <v>551</v>
       </c>
-      <c r="E67" s="19" t="s">
+      <c r="E67" s="20" t="s">
         <v>507</v>
       </c>
-      <c r="F67" s="19" t="s">
+      <c r="F67" s="20" t="s">
         <v>532</v>
       </c>
       <c r="G67" s="5" t="s">
@@ -7842,13 +7843,13 @@
       <c r="C68" s="5" t="s">
         <v>556</v>
       </c>
-      <c r="D68" s="19" t="s">
+      <c r="D68" s="20" t="s">
         <v>522</v>
       </c>
-      <c r="E68" s="19" t="s">
+      <c r="E68" s="20" t="s">
         <v>512</v>
       </c>
-      <c r="F68" s="19" t="s">
+      <c r="F68" s="20" t="s">
         <v>559</v>
       </c>
       <c r="G68" s="5" t="s">
@@ -7861,13 +7862,13 @@
       <c r="C69" s="5" t="s">
         <v>556</v>
       </c>
-      <c r="D69" s="19" t="s">
+      <c r="D69" s="20" t="s">
         <v>560</v>
       </c>
-      <c r="E69" s="19" t="s">
+      <c r="E69" s="20" t="s">
         <v>561</v>
       </c>
-      <c r="F69" s="19" t="s">
+      <c r="F69" s="20" t="s">
         <v>562</v>
       </c>
       <c r="G69" s="5" t="s">
@@ -7880,13 +7881,13 @@
       <c r="C70" s="5" t="s">
         <v>556</v>
       </c>
-      <c r="D70" s="19" t="s">
+      <c r="D70" s="20" t="s">
         <v>510</v>
       </c>
-      <c r="E70" s="19" t="s">
+      <c r="E70" s="20" t="s">
         <v>559</v>
       </c>
-      <c r="F70" s="19" t="s">
+      <c r="F70" s="20" t="s">
         <v>563</v>
       </c>
       <c r="G70" s="5" t="s">
@@ -7899,13 +7900,13 @@
       <c r="C71" s="5" t="s">
         <v>556</v>
       </c>
-      <c r="D71" s="19" t="s">
+      <c r="D71" s="20" t="s">
         <v>563</v>
       </c>
-      <c r="E71" s="19" t="s">
+      <c r="E71" s="20" t="s">
         <v>564</v>
       </c>
-      <c r="F71" s="19" t="s">
+      <c r="F71" s="20" t="s">
         <v>565</v>
       </c>
       <c r="G71" s="5" t="s">
@@ -7918,13 +7919,13 @@
       <c r="C72" s="5" t="s">
         <v>556</v>
       </c>
-      <c r="D72" s="19" t="s">
+      <c r="D72" s="20" t="s">
         <v>566</v>
       </c>
-      <c r="E72" s="19" t="s">
+      <c r="E72" s="20" t="s">
         <v>542</v>
       </c>
-      <c r="F72" s="19" t="s">
+      <c r="F72" s="20" t="s">
         <v>567</v>
       </c>
       <c r="G72" s="5" t="s">
@@ -7935,16 +7936,16 @@
       <c r="A73" s="5"/>
       <c r="B73" s="5"/>
       <c r="C73" s="5"/>
-      <c r="D73" s="20" t="s">
+      <c r="D73" s="21" t="s">
         <v>568</v>
       </c>
-      <c r="E73" s="20" t="s">
+      <c r="E73" s="21" t="s">
         <v>569</v>
       </c>
-      <c r="F73" s="20" t="s">
+      <c r="F73" s="21" t="s">
         <v>570</v>
       </c>
-      <c r="G73" s="23" t="s">
+      <c r="G73" s="24" t="s">
         <v>455</v>
       </c>
     </row>
@@ -7954,13 +7955,13 @@
       <c r="C74" s="5" t="s">
         <v>571</v>
       </c>
-      <c r="D74" s="19" t="s">
+      <c r="D74" s="20" t="s">
         <v>572</v>
       </c>
-      <c r="E74" s="19" t="s">
+      <c r="E74" s="20" t="s">
         <v>510</v>
       </c>
-      <c r="F74" s="19" t="s">
+      <c r="F74" s="20" t="s">
         <v>573</v>
       </c>
       <c r="G74" s="5" t="s">
@@ -7973,13 +7974,13 @@
       <c r="C75" s="5" t="s">
         <v>571</v>
       </c>
-      <c r="D75" s="19" t="s">
+      <c r="D75" s="20" t="s">
         <v>574</v>
       </c>
-      <c r="E75" s="19" t="s">
+      <c r="E75" s="20" t="s">
         <v>575</v>
       </c>
-      <c r="F75" s="19" t="s">
+      <c r="F75" s="20" t="s">
         <v>576</v>
       </c>
       <c r="G75" s="5" t="s">
@@ -7992,13 +7993,13 @@
       <c r="C76" s="5" t="s">
         <v>571</v>
       </c>
-      <c r="D76" s="19" t="s">
+      <c r="D76" s="20" t="s">
         <v>577</v>
       </c>
-      <c r="E76" s="19" t="s">
+      <c r="E76" s="20" t="s">
         <v>578</v>
       </c>
-      <c r="F76" s="19" t="s">
+      <c r="F76" s="20" t="s">
         <v>579</v>
       </c>
       <c r="G76" s="5" t="s">
@@ -8011,13 +8012,13 @@
       <c r="C77" s="5" t="s">
         <v>571</v>
       </c>
-      <c r="D77" s="19" t="s">
+      <c r="D77" s="20" t="s">
         <v>580</v>
       </c>
-      <c r="E77" s="19" t="s">
+      <c r="E77" s="20" t="s">
         <v>581</v>
       </c>
-      <c r="F77" s="19" t="s">
+      <c r="F77" s="20" t="s">
         <v>582</v>
       </c>
       <c r="G77" s="5" t="s">
@@ -8030,13 +8031,13 @@
       <c r="C78" s="5" t="s">
         <v>571</v>
       </c>
-      <c r="D78" s="19" t="s">
+      <c r="D78" s="20" t="s">
         <v>583</v>
       </c>
-      <c r="E78" s="19" t="s">
+      <c r="E78" s="20" t="s">
         <v>583</v>
       </c>
-      <c r="F78" s="19" t="s">
+      <c r="F78" s="20" t="s">
         <v>584</v>
       </c>
       <c r="G78" s="5" t="s">
@@ -8049,13 +8050,13 @@
       <c r="C79" s="5" t="s">
         <v>571</v>
       </c>
-      <c r="D79" s="19" t="s">
+      <c r="D79" s="20" t="s">
         <v>585</v>
       </c>
-      <c r="E79" s="19" t="s">
+      <c r="E79" s="20" t="s">
         <v>586</v>
       </c>
-      <c r="F79" s="19" t="s">
+      <c r="F79" s="20" t="s">
         <v>587</v>
       </c>
       <c r="G79" s="5" t="s">
@@ -8068,13 +8069,13 @@
       <c r="C80" s="5" t="s">
         <v>571</v>
       </c>
-      <c r="D80" s="19" t="s">
+      <c r="D80" s="20" t="s">
         <v>588</v>
       </c>
-      <c r="E80" s="19" t="s">
+      <c r="E80" s="20" t="s">
         <v>589</v>
       </c>
-      <c r="F80" s="19" t="s">
+      <c r="F80" s="20" t="s">
         <v>590</v>
       </c>
       <c r="G80" s="5" t="s">
@@ -8087,13 +8088,13 @@
       <c r="C81" s="5" t="s">
         <v>571</v>
       </c>
-      <c r="D81" s="19" t="s">
+      <c r="D81" s="20" t="s">
         <v>591</v>
       </c>
-      <c r="E81" s="19" t="s">
+      <c r="E81" s="20" t="s">
         <v>592</v>
       </c>
-      <c r="F81" s="19" t="s">
+      <c r="F81" s="20" t="s">
         <v>593</v>
       </c>
       <c r="G81" s="5" t="s">
@@ -8104,16 +8105,16 @@
       <c r="A82" s="5"/>
       <c r="B82" s="5"/>
       <c r="C82" s="5"/>
-      <c r="D82" s="20" t="s">
+      <c r="D82" s="21" t="s">
         <v>594</v>
       </c>
-      <c r="E82" s="20" t="s">
+      <c r="E82" s="21" t="s">
         <v>570</v>
       </c>
-      <c r="F82" s="22">
+      <c r="F82" s="23">
         <v>1259</v>
       </c>
-      <c r="G82" s="23" t="s">
+      <c r="G82" s="24" t="s">
         <v>455</v>
       </c>
     </row>
@@ -8244,7 +8245,7 @@
       <c r="D6" s="4" t="s">
         <v>624</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="E6" s="7" t="s">
         <v>625</v>
       </c>
       <c r="F6" s="5" t="s">
@@ -8256,7 +8257,7 @@
       <c r="H6" s="5" t="s">
         <v>628</v>
       </c>
-      <c r="I6" s="10" t="s">
+      <c r="I6" s="11" t="s">
         <v>629</v>
       </c>
     </row>
@@ -8278,18 +8279,18 @@
       <c r="B9" s="5" t="s">
         <v>633</v>
       </c>
-      <c r="F9" s="7" t="s">
+      <c r="F9" s="8" t="s">
         <v>634</v>
       </c>
-      <c r="G9" s="7" t="s">
+      <c r="G9" s="8" t="s">
         <v>635</v>
       </c>
     </row>
     <row r="10" spans="6:7">
-      <c r="F10" s="7" t="s">
+      <c r="F10" s="8" t="s">
         <v>636</v>
       </c>
-      <c r="G10" s="7" t="s">
+      <c r="G10" s="8" t="s">
         <v>637</v>
       </c>
     </row>
@@ -8297,10 +8298,10 @@
       <c r="A11" s="2" t="s">
         <v>638</v>
       </c>
-      <c r="F11" s="7" t="s">
+      <c r="F11" s="8" t="s">
         <v>639</v>
       </c>
-      <c r="G11" s="7" t="s">
+      <c r="G11" s="8" t="s">
         <v>640</v>
       </c>
     </row>
@@ -8309,10 +8310,10 @@
         <v>641</v>
       </c>
       <c r="B12" s="5"/>
-      <c r="F12" s="7" t="s">
+      <c r="F12" s="8" t="s">
         <v>642</v>
       </c>
-      <c r="G12" s="7" t="s">
+      <c r="G12" s="8" t="s">
         <v>643</v>
       </c>
     </row>
@@ -8323,10 +8324,10 @@
       <c r="B13" s="5" t="s">
         <v>644</v>
       </c>
-      <c r="F13" s="7" t="s">
+      <c r="F13" s="8" t="s">
         <v>645</v>
       </c>
-      <c r="G13" s="7" t="s">
+      <c r="G13" s="8" t="s">
         <v>646</v>
       </c>
     </row>
@@ -8337,27 +8338,27 @@
       <c r="B14" s="5" t="s">
         <v>648</v>
       </c>
-      <c r="F14" s="7" t="s">
+      <c r="F14" s="8" t="s">
         <v>649</v>
       </c>
-      <c r="G14" s="8" t="s">
+      <c r="G14" s="9" t="s">
         <v>650</v>
       </c>
     </row>
     <row r="15" spans="6:7">
-      <c r="F15" s="7" t="s">
+      <c r="F15" s="8" t="s">
         <v>651</v>
       </c>
-      <c r="G15" s="7"/>
+      <c r="G15" s="8"/>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" s="2" t="s">
         <v>652</v>
       </c>
-      <c r="F16" s="7" t="s">
+      <c r="F16" s="8" t="s">
         <v>653</v>
       </c>
-      <c r="G16" s="7" t="s">
+      <c r="G16" s="8" t="s">
         <v>654</v>
       </c>
     </row>
@@ -8453,7 +8454,7 @@
       </c>
     </row>
     <row r="47" ht="185" spans="5:5">
-      <c r="E47" s="9" t="s">
+      <c r="E47" s="10" t="s">
         <v>673</v>
       </c>
     </row>

</xml_diff>